<commit_message>
Adding content from stream.
</commit_message>
<xml_diff>
--- a/_Projects/P1012202501-ESP32_Stepper_Controller/ProjectDocuments/P1012202501-ECR_ECN.xlsx
+++ b/_Projects/P1012202501-ESP32_Stepper_Controller/ProjectDocuments/P1012202501-ECR_ECN.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
+  <workbookPr backupFile="false" showObjects="all" dateCompatibility="false"/>
   <workbookProtection/>
   <bookViews>
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="41">
   <si>
     <t xml:space="preserve">ENGINEERING CHANGE REQUEST</t>
   </si>
@@ -31,7 +31,7 @@
     <t xml:space="preserve">ECR No:</t>
   </si>
   <si>
-    <t xml:space="preserve">P1012202501-01-11-26-01</t>
+    <t xml:space="preserve">P1012202501-01-17-26-01</t>
   </si>
   <si>
     <t xml:space="preserve">Customer Name:</t>
@@ -64,13 +64,13 @@
     <t xml:space="preserve">CHANGE REQUESTED</t>
   </si>
   <si>
-    <t xml:space="preserve">Replace IC5 with CP2102N-A02-GQFN28R for proper USB to UART functionality.</t>
+    <t xml:space="preserve">Add 100nF capacitor between TEMP_SENSE line and GND on the ESP32 to better filter out noise on the analog line.</t>
   </si>
   <si>
     <t xml:space="preserve">REASON FOR CHANGE</t>
   </si>
   <si>
-    <t xml:space="preserve">Bench testing had a failure of the original part #CP2102C-A01-GQFN28 even after replacement.</t>
+    <t xml:space="preserve">Bench testing has a lot of signal noise on that line, the capacitor should help to stabilize it better.</t>
   </si>
   <si>
     <t xml:space="preserve">REQUESTED BY</t>
@@ -106,7 +106,7 @@
     <t xml:space="preserve">Can this change be done and does it provide value to the customer or company or is the change necessary for product/service operation?</t>
   </si>
   <si>
-    <t xml:space="preserve">It can be done and is necessary for the proper operation of the device.</t>
+    <t xml:space="preserve">It can be done and will help the proper operation of the device.</t>
   </si>
   <si>
     <t xml:space="preserve">REVIEWED BY</t>
@@ -136,7 +136,7 @@
     <t xml:space="preserve">ECN No:</t>
   </si>
   <si>
-    <t xml:space="preserve">ECN-P1012202501-01-11-26-01</t>
+    <t xml:space="preserve">ECN-P1012202501-01-17-26-01</t>
   </si>
   <si>
     <t xml:space="preserve">ECN Date:</t>
@@ -860,7 +860,7 @@
       </c>
       <c r="D26" s="4"/>
       <c r="E26" s="8" t="n">
-        <v>46031</v>
+        <v>46039</v>
       </c>
       <c r="F26" s="8"/>
       <c r="G26" s="4"/>
@@ -1066,7 +1066,7 @@
       </c>
       <c r="D46" s="4"/>
       <c r="E46" s="8" t="n">
-        <v>46033</v>
+        <v>46039</v>
       </c>
       <c r="F46" s="8"/>
       <c r="G46" s="4"/>
@@ -1260,12 +1260,14 @@
       </c>
       <c r="D60" s="4"/>
       <c r="E60" s="8" t="n">
-        <v>46033</v>
+        <v>46039</v>
       </c>
       <c r="F60" s="8"/>
       <c r="G60" s="4"/>
       <c r="H60" s="4"/>
-      <c r="I60" s="4"/>
+      <c r="I60" s="4" t="s">
+        <v>25</v>
+      </c>
       <c r="J60" s="4"/>
     </row>
     <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1344,7 +1346,7 @@
       </c>
       <c r="F66" s="3"/>
       <c r="G66" s="14" t="n">
-        <v>46033</v>
+        <v>46039</v>
       </c>
       <c r="H66" s="14"/>
       <c r="I66" s="13"/>

</xml_diff>